<commit_message>
Adicionar exportacao de encomendas selecionadas
</commit_message>
<xml_diff>
--- a/public/ATT_IMPORT.xlsx
+++ b/public/ATT_IMPORT.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ezcle\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\trilhos-model-export\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{938D5A3D-B037-42A1-8173-67424BE6C6CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5CFC4833-6682-4A31-B346-425952DA1958}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3855" yWindow="3855" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Folha1" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
   <si>
     <t>REF</t>
   </si>
@@ -74,15 +74,6 @@
   </si>
   <si>
     <t>SERVIÇO</t>
-  </si>
-  <si>
-    <t>600 83 40 57</t>
-  </si>
-  <si>
-    <t>619 725 043</t>
-  </si>
-  <si>
-    <t>+34</t>
   </si>
 </sst>
 </file>
@@ -597,253 +588,95 @@
     <col min="2" max="2" width="16.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B1" s="2">
-        <v>722155691</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B2" s="2">
-        <v>653616339</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B3" s="2">
-        <v>643421054</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B4" s="3">
-        <v>625148290</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B5" s="2">
-        <v>685775642</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B6" s="2">
-        <v>684661638</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B7" s="2">
-        <v>656467122</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B8" s="2">
-        <v>634811636</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B9" s="2">
-        <v>643424450</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B10" s="2">
-        <v>653983432</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A11" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B11" s="2">
-        <v>691038370</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A12" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B12" s="2">
-        <v>642965738</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A13" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B13" s="2">
-        <v>642571538</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A14" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B14" s="2">
-        <v>689619305</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A15" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B15" s="2">
-        <v>659898963</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A16" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B16" s="2">
-        <v>642768089</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A17" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B17" s="2">
-        <v>653344081</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A18" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B18" s="4">
-        <v>65249789</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A19" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B19" s="2">
-        <v>699514856</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A20" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B20" s="2">
-        <v>624227372</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A21" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B21" s="2">
-        <v>642169300</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A22" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B22" s="2" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A23" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B23" s="2">
-        <v>675433793</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A24" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B24" s="2">
-        <v>686704428</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A25" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B25" s="2">
-        <v>601385725</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A26" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B26" s="2">
-        <v>637016901</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A27" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B27" s="2">
-        <v>693816639</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A28" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B28" s="2">
-        <v>626833766</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A29" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B29" s="2">
-        <v>611811125</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A30" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B30" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="31" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A31" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B31" s="2">
-        <v>603325109</v>
-      </c>
+    <row r="1" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B1" s="2"/>
+    </row>
+    <row r="2" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B2" s="2"/>
+    </row>
+    <row r="3" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B3" s="2"/>
+    </row>
+    <row r="4" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B4" s="3"/>
+    </row>
+    <row r="5" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B5" s="2"/>
+    </row>
+    <row r="6" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B6" s="2"/>
+    </row>
+    <row r="7" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B7" s="2"/>
+    </row>
+    <row r="9" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B9" s="2"/>
+    </row>
+    <row r="10" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B10" s="2"/>
+    </row>
+    <row r="11" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B11" s="2"/>
+    </row>
+    <row r="12" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B12" s="2"/>
+    </row>
+    <row r="13" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B13" s="2"/>
+    </row>
+    <row r="14" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B14" s="2"/>
+    </row>
+    <row r="15" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B15" s="2"/>
+    </row>
+    <row r="16" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B16" s="2"/>
+    </row>
+    <row r="17" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B17" s="2"/>
+    </row>
+    <row r="18" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B18" s="4"/>
+    </row>
+    <row r="19" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B19" s="2"/>
+    </row>
+    <row r="20" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B20" s="2"/>
+    </row>
+    <row r="21" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B21" s="2"/>
+    </row>
+    <row r="22" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B22" s="2"/>
+    </row>
+    <row r="23" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B23" s="2"/>
+    </row>
+    <row r="24" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B24" s="2"/>
+    </row>
+    <row r="25" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B25" s="2"/>
+    </row>
+    <row r="26" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B26" s="2"/>
+    </row>
+    <row r="27" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B27" s="2"/>
+    </row>
+    <row r="28" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B28" s="2"/>
+    </row>
+    <row r="29" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B29" s="2"/>
+    </row>
+    <row r="30" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B30" s="2"/>
+    </row>
+    <row r="31" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B31" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>